<commit_message>
Set BHP to 9000 units; scheduled task mirrors EOD shortcut
- Change BHP.AX holding 10000 -> 9000 in Tickers_and_Shares.txt and the
  inline TICKERS_AND_SHARES fallback in asx_eod_downloader.py
- Rewrite CreateScheduledTask.ps1 to run wscript.exe "run_eod_hidden.vbs"
  (same as the "Run EOD + Open Report" shortcut: download, report, open
  Notepad++) under an interactive, logged-on-only principal
- Update CLAUDE.md scheduled-task docs to match the new action
- Refresh DailyData.csv and reports with the 9000-share BHP figure

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260605.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260605.xlsx
@@ -688,13 +688,13 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2650</v>
+        <v>3000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>259461.5</v>
+        <v>293730</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>14098</v>
+        <v>15960</v>
       </c>
     </row>
     <row r="12">
@@ -731,24 +731,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.002</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>700000</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-1400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1333356.18</v>
+        <v>1369024.68</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-8275.700000000001</v>
+        <v>-5013.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>